<commit_message>
clean file names, file organization for DATA files
</commit_message>
<xml_diff>
--- a/1-data/Particle Density_DELUGE.xlsx
+++ b/1-data/Particle Density_DELUGE.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30006"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pnnl-my.sharepoint.com/personal/marci_garcia_pnnl_gov/Documents/Kenton pH water/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="161" documentId="8_{149C9F74-8D7B-4648-A146-1D621F11431C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2361381-999D-4E2F-AE52-0A34009E6B99}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{25CE4122-9A44-4115-916F-2EB8F45536C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{318262BB-F1FF-485E-8DD9-B44390E1733D}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
   <si>
     <t>Label ID</t>
   </si>
@@ -125,6 +125,27 @@
   </si>
   <si>
     <t>water</t>
+  </si>
+  <si>
+    <t>Ground samples</t>
+  </si>
+  <si>
+    <t>g water</t>
+  </si>
+  <si>
+    <t>ml</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>g/ml</t>
+  </si>
+  <si>
+    <t>former value</t>
+  </si>
+  <si>
+    <t>difference</t>
   </si>
   <si>
     <t>#</t>
@@ -303,7 +324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -326,7 +347,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -339,6 +359,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -792,7 +816,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EA15916-E3CF-4D1E-ACAA-B47F7C195023}">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.42578125" style="2" customWidth="1"/>
@@ -801,28 +825,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" ht="57.75">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="D1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="E1" s="21" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="19" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="9" t="s">
@@ -857,7 +881,7 @@
       <c r="H2" s="12">
         <v>0.99799199999999999</v>
       </c>
-      <c r="I2" s="15">
+      <c r="I2" s="25">
         <f>(D2-C2)/(F2-((E2-D2)/H2))</f>
         <v>3.1872931760369676</v>
       </c>
@@ -887,8 +911,8 @@
       <c r="H3" s="12">
         <v>0.99799199999999999</v>
       </c>
-      <c r="I3" s="15">
-        <f t="shared" ref="I3:I19" si="0">(D3-C3)/(F3-((E3-D3)/H3))</f>
+      <c r="I3" s="25">
+        <f t="shared" ref="I3:I38" si="0">(D3-C3)/(F3-((E3-D3)/H3))</f>
         <v>2.3958757110784039</v>
       </c>
     </row>
@@ -918,12 +942,12 @@
         <v>0.99799199999999999</v>
       </c>
       <c r="I4">
-        <f t="shared" si="0"/>
+        <f>(D4-C4)/(F4-((E4-D4)/H4))</f>
         <v>2.8435521548919076</v>
       </c>
       <c r="J4">
-        <f>AVERAGE(I4:I7,I11,I12,I13)</f>
-        <v>2.7630085449624979</v>
+        <f>AVERAGE(I2:I7,I11,I12,I13,I14,I15,I16,I17,I19,I8)</f>
+        <v>2.7847580662129325</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1032,8 +1056,8 @@
       <c r="E8" s="4">
         <v>47.5929</v>
       </c>
-      <c r="F8" s="18">
-        <v>25</v>
+      <c r="F8" s="23">
+        <v>24.59</v>
       </c>
       <c r="G8" s="12">
         <v>21</v>
@@ -1041,9 +1065,9 @@
       <c r="H8" s="12">
         <v>0.99799199999999999</v>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="25">
         <f t="shared" si="0"/>
-        <v>1.8711872948374784</v>
+        <v>3.0734773238817614</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1062,8 +1086,8 @@
       <c r="E9" s="4">
         <v>49.546100000000003</v>
       </c>
-      <c r="F9" s="18">
-        <v>25</v>
+      <c r="F9" s="23">
+        <v>25.307081135999997</v>
       </c>
       <c r="G9" s="12">
         <v>21</v>
@@ -1073,7 +1097,7 @@
       </c>
       <c r="I9" s="15">
         <f>(D9-C9)/(F9-((E9-D9)/H9))</f>
-        <v>14.180287327787294</v>
+        <v>3.9948729471796596</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -1092,8 +1116,8 @@
       <c r="E10" s="4">
         <v>48.521599999999999</v>
       </c>
-      <c r="F10" s="18">
-        <v>25</v>
+      <c r="F10" s="23">
+        <v>25.235924306400001</v>
       </c>
       <c r="G10" s="12">
         <v>21</v>
@@ -1103,7 +1127,7 @@
       </c>
       <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v>2.3343506051860685</v>
+        <v>1.859369910753907</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -1122,8 +1146,8 @@
       <c r="E11" s="4">
         <v>48.472000000000001</v>
       </c>
-      <c r="F11" s="17">
-        <v>25.075959514981463</v>
+      <c r="F11" s="16">
+        <v>24.973053213600004</v>
       </c>
       <c r="G11" s="12">
         <v>21</v>
@@ -1132,8 +1156,8 @@
         <v>0.99799199999999999</v>
       </c>
       <c r="I11">
-        <f t="shared" si="0"/>
-        <v>2.8275854202987496</v>
+        <f>(D11-C11)/(F11-((E11-D11)/H11))</f>
+        <v>3.1894414042706911</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -1152,8 +1176,8 @@
       <c r="E12" s="4">
         <v>48.037999999999997</v>
       </c>
-      <c r="F12" s="17">
-        <v>25.095400340715507</v>
+      <c r="F12" s="16">
+        <v>24.992414258400004</v>
       </c>
       <c r="G12" s="12">
         <v>21</v>
@@ -1163,7 +1187,7 @@
       </c>
       <c r="I12">
         <f t="shared" si="0"/>
-        <v>2.5645238242585142</v>
+        <v>2.9033026642057265</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -1182,8 +1206,8 @@
       <c r="E13" s="4">
         <v>49.673299999999998</v>
       </c>
-      <c r="F13" s="17">
-        <v>25.262350936967632</v>
+      <c r="F13" s="16">
+        <v>25.158679725599999</v>
       </c>
       <c r="G13" s="12">
         <v>21</v>
@@ -1193,7 +1217,7 @@
       </c>
       <c r="I13">
         <f t="shared" si="0"/>
-        <v>2.7194738676302328</v>
+        <v>3.0249862648370196</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -1225,10 +1249,6 @@
         <f t="shared" si="0"/>
         <v>2.5871549181476534</v>
       </c>
-      <c r="J14">
-        <f>AVERAGE(I14:I17,I19)</f>
-        <v>2.5535035492666864</v>
-      </c>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="6" t="s">
@@ -1290,7 +1310,7 @@
         <v>2.5144431147166282</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:14">
       <c r="A17" s="6" t="s">
         <v>25</v>
       </c>
@@ -1320,7 +1340,7 @@
         <v>2.5142778194056072</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:14">
       <c r="A18" s="6" t="s">
         <v>26</v>
       </c>
@@ -1350,7 +1370,7 @@
         <v>1.4157145923287719</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:14">
       <c r="A19" s="6" t="s">
         <v>27</v>
       </c>
@@ -1380,7 +1400,7 @@
         <v>2.6002358643823138</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:14">
       <c r="A20" s="8" t="s">
         <v>28</v>
       </c>
@@ -1396,7 +1416,10 @@
       <c r="E20" s="4">
         <v>46.810200000000002</v>
       </c>
-      <c r="F20" s="16"/>
+      <c r="F20" s="16">
+        <f>(E20-C20)*H20</f>
+        <v>24.973053213600004</v>
+      </c>
       <c r="G20" s="12">
         <v>21</v>
       </c>
@@ -1404,7 +1427,7 @@
         <v>0.99799199999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:14">
       <c r="A21" s="8" t="s">
         <v>28</v>
       </c>
@@ -1420,7 +1443,10 @@
       <c r="E21" s="4">
         <v>46.653100000000002</v>
       </c>
-      <c r="F21" s="16"/>
+      <c r="F21" s="16">
+        <f t="shared" ref="F21:F25" si="1">(E21-C21)*H21</f>
+        <v>24.992414258400004</v>
+      </c>
       <c r="G21" s="12">
         <v>21</v>
       </c>
@@ -1428,7 +1454,7 @@
         <v>0.99799199999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:14">
       <c r="A22" s="8" t="s">
         <v>28</v>
       </c>
@@ -1444,7 +1470,10 @@
       <c r="E22" s="4">
         <v>47.9039</v>
       </c>
-      <c r="F22" s="16"/>
+      <c r="F22" s="16">
+        <f t="shared" si="1"/>
+        <v>25.158679725599999</v>
+      </c>
       <c r="G22" s="12">
         <v>21</v>
       </c>
@@ -1452,7 +1481,7 @@
         <v>0.99799199999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:14">
       <c r="A23" s="8" t="s">
         <v>28</v>
       </c>
@@ -1468,8 +1497,15 @@
       <c r="E23">
         <v>45.906799999999997</v>
       </c>
-    </row>
-    <row r="24" spans="1:9">
+      <c r="F23" s="16"/>
+      <c r="G23" s="12">
+        <v>21</v>
+      </c>
+      <c r="H23" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
       <c r="A24" s="8" t="s">
         <v>28</v>
       </c>
@@ -1485,8 +1521,18 @@
       <c r="E24">
         <v>48.366599999999998</v>
       </c>
-    </row>
-    <row r="25" spans="1:9">
+      <c r="F24" s="16">
+        <f t="shared" si="1"/>
+        <v>25.307081135999997</v>
+      </c>
+      <c r="G24" s="12">
+        <v>21</v>
+      </c>
+      <c r="H24" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
       <c r="A25" s="8" t="s">
         <v>28</v>
       </c>
@@ -1501,6 +1547,1022 @@
       </c>
       <c r="E25">
         <v>47.624299999999998</v>
+      </c>
+      <c r="F25" s="16">
+        <f t="shared" si="1"/>
+        <v>25.235924306400001</v>
+      </c>
+      <c r="G25" s="12">
+        <v>21</v>
+      </c>
+      <c r="H25" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
+      <c r="A26" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K26" t="s">
+        <v>30</v>
+      </c>
+      <c r="L26" t="s">
+        <v>31</v>
+      </c>
+      <c r="M26" t="s">
+        <v>32</v>
+      </c>
+      <c r="N26" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
+      <c r="A27" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27">
+        <v>23.1129</v>
+      </c>
+      <c r="D27">
+        <v>23.534800000000001</v>
+      </c>
+      <c r="E27">
+        <v>47.664499999999997</v>
+      </c>
+      <c r="F27" s="12">
+        <v>24.31</v>
+      </c>
+      <c r="G27">
+        <v>21</v>
+      </c>
+      <c r="H27" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I27" s="25">
+        <f>(D27-C27)/(F27-((E27-D27)/H27))</f>
+        <v>3.202275237607858</v>
+      </c>
+      <c r="K27">
+        <f>E27-D27</f>
+        <v>24.129699999999996</v>
+      </c>
+      <c r="L27">
+        <f>F27-K27</f>
+        <v>0.18030000000000257</v>
+      </c>
+      <c r="M27">
+        <f>D27-C27</f>
+        <v>0.42190000000000083</v>
+      </c>
+      <c r="N27">
+        <f>M27/L27</f>
+        <v>2.3399889073765658</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
+      <c r="A28" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28">
+        <v>2</v>
+      </c>
+      <c r="C28">
+        <v>19.6692</v>
+      </c>
+      <c r="D28">
+        <v>19.951499999999999</v>
+      </c>
+      <c r="E28">
+        <v>45.415500000000002</v>
+      </c>
+      <c r="F28" s="12">
+        <v>25.65</v>
+      </c>
+      <c r="G28">
+        <v>21</v>
+      </c>
+      <c r="H28" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I28" s="25">
+        <f t="shared" ref="I28:I38" si="2">(D28-C28)/(F28-((E28-D28)/H28))</f>
+        <v>2.0947511844324764</v>
+      </c>
+      <c r="K28">
+        <f t="shared" ref="K28:K34" si="3">E28-D28</f>
+        <v>25.464000000000002</v>
+      </c>
+      <c r="L28">
+        <f t="shared" ref="L28:L34" si="4">F28-K28</f>
+        <v>0.18599999999999639</v>
+      </c>
+      <c r="M28">
+        <f t="shared" ref="M28:M38" si="5">D28-C28</f>
+        <v>0.28229999999999933</v>
+      </c>
+      <c r="N28">
+        <f t="shared" ref="N28:N38" si="6">M28/L28</f>
+        <v>1.5177419354838968</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14">
+      <c r="A29" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29">
+        <v>23.3216</v>
+      </c>
+      <c r="D29">
+        <v>23.943100000000001</v>
+      </c>
+      <c r="E29">
+        <v>48.505800000000001</v>
+      </c>
+      <c r="F29" s="12">
+        <v>24.87</v>
+      </c>
+      <c r="G29">
+        <v>21</v>
+      </c>
+      <c r="H29" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I29" s="25">
+        <f t="shared" si="2"/>
+        <v>2.4100463224736677</v>
+      </c>
+      <c r="J29">
+        <f>AVERAGE(I27:I29)</f>
+        <v>2.5690242481713339</v>
+      </c>
+      <c r="K29">
+        <f t="shared" si="3"/>
+        <v>24.5627</v>
+      </c>
+      <c r="L29">
+        <f t="shared" si="4"/>
+        <v>0.30730000000000146</v>
+      </c>
+      <c r="M29">
+        <f t="shared" si="5"/>
+        <v>0.62150000000000105</v>
+      </c>
+      <c r="N29">
+        <f t="shared" si="6"/>
+        <v>2.0224536283761734</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
+      <c r="A30" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30">
+        <v>4</v>
+      </c>
+      <c r="C30">
+        <v>19.913599999999999</v>
+      </c>
+      <c r="D30">
+        <v>20.1938</v>
+      </c>
+      <c r="E30">
+        <v>45.375599999999999</v>
+      </c>
+      <c r="F30" s="12">
+        <v>25.36</v>
+      </c>
+      <c r="G30">
+        <v>21</v>
+      </c>
+      <c r="H30" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I30" s="25">
+        <f t="shared" si="2"/>
+        <v>2.1970748426740085</v>
+      </c>
+      <c r="K30">
+        <f t="shared" si="3"/>
+        <v>25.181799999999999</v>
+      </c>
+      <c r="L30">
+        <f t="shared" si="4"/>
+        <v>0.17820000000000036</v>
+      </c>
+      <c r="M30">
+        <f t="shared" si="5"/>
+        <v>0.28020000000000067</v>
+      </c>
+      <c r="N30">
+        <f t="shared" si="6"/>
+        <v>1.5723905723905729</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
+      <c r="A31" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31">
+        <v>5</v>
+      </c>
+      <c r="C31">
+        <v>23.1782</v>
+      </c>
+      <c r="D31">
+        <v>23.505400000000002</v>
+      </c>
+      <c r="E31">
+        <v>48.672899999999998</v>
+      </c>
+      <c r="F31" s="12">
+        <v>25.36</v>
+      </c>
+      <c r="G31">
+        <v>21</v>
+      </c>
+      <c r="H31" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I31" s="25">
+        <f t="shared" si="2"/>
+        <v>2.3064671918739013</v>
+      </c>
+      <c r="K31">
+        <f t="shared" si="3"/>
+        <v>25.167499999999997</v>
+      </c>
+      <c r="L31">
+        <f t="shared" si="4"/>
+        <v>0.19250000000000256</v>
+      </c>
+      <c r="M31">
+        <f t="shared" si="5"/>
+        <v>0.32720000000000127</v>
+      </c>
+      <c r="N31">
+        <f t="shared" si="6"/>
+        <v>1.6997402597402438</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
+      <c r="A32" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B32">
+        <v>6</v>
+      </c>
+      <c r="C32">
+        <v>19.669699999999999</v>
+      </c>
+      <c r="D32">
+        <v>20.086200000000002</v>
+      </c>
+      <c r="E32">
+        <v>44.538200000000003</v>
+      </c>
+      <c r="F32" s="12">
+        <v>24.68</v>
+      </c>
+      <c r="G32">
+        <v>21</v>
+      </c>
+      <c r="H32" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I32" s="25">
+        <f t="shared" si="2"/>
+        <v>2.3293975831775158</v>
+      </c>
+      <c r="J32">
+        <f>AVERAGE(I30:I32)</f>
+        <v>2.2776465392418088</v>
+      </c>
+      <c r="K32">
+        <f t="shared" si="3"/>
+        <v>24.452000000000002</v>
+      </c>
+      <c r="L32">
+        <f t="shared" si="4"/>
+        <v>0.22799999999999798</v>
+      </c>
+      <c r="M32">
+        <f t="shared" si="5"/>
+        <v>0.41650000000000276</v>
+      </c>
+      <c r="N32">
+        <f t="shared" si="6"/>
+        <v>1.8267543859649404</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14">
+      <c r="A33" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B33" s="17">
+        <v>7</v>
+      </c>
+      <c r="C33">
+        <v>21.3018</v>
+      </c>
+      <c r="D33">
+        <v>21.6938</v>
+      </c>
+      <c r="E33">
+        <v>46.137700000000002</v>
+      </c>
+      <c r="F33" s="23">
+        <v>24.130348768799994</v>
+      </c>
+      <c r="G33">
+        <v>21</v>
+      </c>
+      <c r="H33" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I33" s="25">
+        <f t="shared" si="2"/>
+        <v>-1.0806836777654567</v>
+      </c>
+      <c r="K33">
+        <f t="shared" si="3"/>
+        <v>24.443900000000003</v>
+      </c>
+      <c r="L33">
+        <f t="shared" si="4"/>
+        <v>-0.31355123120000883</v>
+      </c>
+      <c r="M33">
+        <f t="shared" si="5"/>
+        <v>0.39199999999999946</v>
+      </c>
+      <c r="N33">
+        <f t="shared" si="6"/>
+        <v>-1.2501944211788139</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
+      <c r="A34" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B34" s="17">
+        <v>8</v>
+      </c>
+      <c r="C34">
+        <v>23.0153</v>
+      </c>
+      <c r="D34">
+        <v>23.2301</v>
+      </c>
+      <c r="E34">
+        <v>48.478999999999999</v>
+      </c>
+      <c r="F34" s="23">
+        <v>25.307081135999997</v>
+      </c>
+      <c r="G34">
+        <v>21</v>
+      </c>
+      <c r="H34" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I34" s="25">
+        <f t="shared" si="2"/>
+        <v>29.108314815896083</v>
+      </c>
+      <c r="K34">
+        <f t="shared" si="3"/>
+        <v>25.248899999999999</v>
+      </c>
+      <c r="L34">
+        <f t="shared" si="4"/>
+        <v>5.818113599999819E-2</v>
+      </c>
+      <c r="M34">
+        <f t="shared" si="5"/>
+        <v>0.21480000000000032</v>
+      </c>
+      <c r="N34">
+        <f t="shared" si="6"/>
+        <v>3.6919182877420442</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
+      <c r="A35" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35" s="17">
+        <v>9</v>
+      </c>
+      <c r="C35">
+        <v>22.7776</v>
+      </c>
+      <c r="D35">
+        <v>23.347000000000001</v>
+      </c>
+      <c r="E35">
+        <v>47.961300000000001</v>
+      </c>
+      <c r="F35" s="23">
+        <v>25.235924306400001</v>
+      </c>
+      <c r="G35">
+        <v>21</v>
+      </c>
+      <c r="H35" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I35" s="25">
+        <f t="shared" si="2"/>
+        <v>0.99528168333224276</v>
+      </c>
+      <c r="J35">
+        <f>AVERAGE(I33:I35)</f>
+        <v>9.6743042738209564</v>
+      </c>
+      <c r="K35">
+        <f t="shared" ref="K35:K38" si="7">E35-D35</f>
+        <v>24.6143</v>
+      </c>
+      <c r="L35">
+        <f t="shared" ref="L35:L38" si="8">F35-K35</f>
+        <v>0.6216243064000011</v>
+      </c>
+      <c r="M35">
+        <f t="shared" si="5"/>
+        <v>0.56940000000000168</v>
+      </c>
+      <c r="N35">
+        <f t="shared" si="6"/>
+        <v>0.91598734820643535</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
+      <c r="A36" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B36" s="17">
+        <v>5131</v>
+      </c>
+      <c r="C36">
+        <v>22.698899999999998</v>
+      </c>
+      <c r="D36">
+        <v>23.172000000000001</v>
+      </c>
+      <c r="E36">
+        <v>48.217700000000001</v>
+      </c>
+      <c r="F36" s="16">
+        <v>25.16</v>
+      </c>
+      <c r="G36">
+        <v>21</v>
+      </c>
+      <c r="H36" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I36" s="25">
+        <f t="shared" si="2"/>
+        <v>7.4029396513444263</v>
+      </c>
+      <c r="K36">
+        <f t="shared" si="7"/>
+        <v>25.0457</v>
+      </c>
+      <c r="L36">
+        <f t="shared" si="8"/>
+        <v>0.11430000000000007</v>
+      </c>
+      <c r="M36">
+        <f t="shared" si="5"/>
+        <v>0.4731000000000023</v>
+      </c>
+      <c r="N36">
+        <f t="shared" si="6"/>
+        <v>4.1391076115485737</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
+      <c r="A37" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B37" s="17">
+        <v>5155</v>
+      </c>
+      <c r="C37">
+        <v>21.792100000000001</v>
+      </c>
+      <c r="D37">
+        <v>22.270299999999999</v>
+      </c>
+      <c r="E37">
+        <v>47.089300000000001</v>
+      </c>
+      <c r="F37" s="16">
+        <f>(E37-C37)*H37</f>
+        <v>25.246403222400001</v>
+      </c>
+      <c r="G37">
+        <v>21</v>
+      </c>
+      <c r="H37" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I37" s="25">
+        <f t="shared" si="2"/>
+        <v>1.2668677357174347</v>
+      </c>
+      <c r="K37">
+        <f t="shared" si="7"/>
+        <v>24.819000000000003</v>
+      </c>
+      <c r="L37">
+        <f t="shared" si="8"/>
+        <v>0.42740322239999884</v>
+      </c>
+      <c r="M37">
+        <f t="shared" si="5"/>
+        <v>0.47819999999999752</v>
+      </c>
+      <c r="N37">
+        <f t="shared" si="6"/>
+        <v>1.1188497768331258</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
+      <c r="A38" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B38" s="17">
+        <v>5167</v>
+      </c>
+      <c r="C38">
+        <v>21.615500000000001</v>
+      </c>
+      <c r="D38">
+        <v>22.050899999999999</v>
+      </c>
+      <c r="E38">
+        <v>46.907299999999999</v>
+      </c>
+      <c r="F38" s="16">
+        <f t="shared" ref="F38" si="9">(E38-C38)*H38</f>
+        <v>25.241014065599998</v>
+      </c>
+      <c r="G38">
+        <v>21</v>
+      </c>
+      <c r="H38" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I38" s="25">
+        <f t="shared" si="2"/>
+        <v>1.3012474904932811</v>
+      </c>
+      <c r="J38">
+        <f>AVERAGE(I36:I38)</f>
+        <v>3.3236849591850475</v>
+      </c>
+      <c r="K38">
+        <f t="shared" si="7"/>
+        <v>24.856400000000001</v>
+      </c>
+      <c r="L38">
+        <f t="shared" si="8"/>
+        <v>0.38461406559999745</v>
+      </c>
+      <c r="M38">
+        <f t="shared" si="5"/>
+        <v>0.43539999999999779</v>
+      </c>
+      <c r="N38">
+        <f t="shared" si="6"/>
+        <v>1.1320438822765735</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14">
+      <c r="B39" s="17"/>
+      <c r="F39" s="17"/>
+      <c r="H39" s="12"/>
+      <c r="I39" t="s">
+        <v>34</v>
+      </c>
+      <c r="J39" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
+      <c r="A40" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40">
+        <v>23.1129</v>
+      </c>
+      <c r="D40">
+        <v>23.1129</v>
+      </c>
+      <c r="E40">
+        <v>47.418700000000001</v>
+      </c>
+      <c r="F40" s="16">
+        <f>(E40-C40)*H40</f>
+        <v>24.256993953600002</v>
+      </c>
+      <c r="G40">
+        <v>21</v>
+      </c>
+      <c r="H40" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I40">
+        <v>24.31</v>
+      </c>
+      <c r="J40" s="24">
+        <f>I40-F40</f>
+        <v>5.300604639999662E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
+      <c r="A41" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41">
+        <v>19.6692</v>
+      </c>
+      <c r="D41">
+        <v>19.6692</v>
+      </c>
+      <c r="E41">
+        <v>45.247399999999999</v>
+      </c>
+      <c r="F41" s="16">
+        <f t="shared" ref="F41:F51" si="10">(E41-C41)*H41</f>
+        <v>25.5268389744</v>
+      </c>
+      <c r="G41">
+        <v>21</v>
+      </c>
+      <c r="H41" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I41">
+        <v>25.65</v>
+      </c>
+      <c r="J41" s="24">
+        <f t="shared" ref="J41:J51" si="11">I41-F41</f>
+        <v>0.1231610255999982</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14">
+      <c r="A42" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B42">
+        <v>3</v>
+      </c>
+      <c r="C42">
+        <v>23.3216</v>
+      </c>
+      <c r="D42">
+        <v>23.3216</v>
+      </c>
+      <c r="E42">
+        <v>48.143900000000002</v>
+      </c>
+      <c r="F42" s="16">
+        <f t="shared" si="10"/>
+        <v>24.772456821600002</v>
+      </c>
+      <c r="G42">
+        <v>21</v>
+      </c>
+      <c r="H42" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I42">
+        <v>24.87</v>
+      </c>
+      <c r="J42" s="24">
+        <f t="shared" si="11"/>
+        <v>9.7543178399998709E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14">
+      <c r="A43" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B43">
+        <v>4</v>
+      </c>
+      <c r="C43">
+        <v>19.913599999999999</v>
+      </c>
+      <c r="D43">
+        <v>19.913599999999999</v>
+      </c>
+      <c r="E43">
+        <v>45.247399999999999</v>
+      </c>
+      <c r="F43" s="16">
+        <f t="shared" si="10"/>
+        <v>25.282929729599999</v>
+      </c>
+      <c r="G43">
+        <v>21</v>
+      </c>
+      <c r="H43" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I43">
+        <v>25.36</v>
+      </c>
+      <c r="J43" s="24">
+        <f t="shared" si="11"/>
+        <v>7.707027040000014E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
+      <c r="A44" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B44">
+        <v>5</v>
+      </c>
+      <c r="C44">
+        <v>23.1782</v>
+      </c>
+      <c r="D44">
+        <v>23.1782</v>
+      </c>
+      <c r="E44">
+        <v>48.495199999999997</v>
+      </c>
+      <c r="F44" s="16">
+        <f t="shared" si="10"/>
+        <v>25.266163463999998</v>
+      </c>
+      <c r="G44">
+        <v>21</v>
+      </c>
+      <c r="H44" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I44">
+        <v>25.36</v>
+      </c>
+      <c r="J44" s="24">
+        <f t="shared" si="11"/>
+        <v>9.3836536000001303E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14">
+      <c r="A45" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B45">
+        <v>6</v>
+      </c>
+      <c r="C45">
+        <v>19.669699999999999</v>
+      </c>
+      <c r="D45">
+        <v>19.669699999999999</v>
+      </c>
+      <c r="E45">
+        <v>44.280700000000003</v>
+      </c>
+      <c r="F45" s="16">
+        <f t="shared" si="10"/>
+        <v>24.561581112000002</v>
+      </c>
+      <c r="G45">
+        <v>21</v>
+      </c>
+      <c r="H45" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I45">
+        <v>24.68</v>
+      </c>
+      <c r="J45" s="24">
+        <f t="shared" si="11"/>
+        <v>0.11841888799999722</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14">
+      <c r="A46" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B46">
+        <v>7</v>
+      </c>
+      <c r="C46">
+        <v>21.3018</v>
+      </c>
+      <c r="D46">
+        <v>21.3018</v>
+      </c>
+      <c r="E46">
+        <v>45.936399999999999</v>
+      </c>
+      <c r="F46" s="16">
+        <f t="shared" si="10"/>
+        <v>24.585133723199998</v>
+      </c>
+      <c r="G46">
+        <v>21</v>
+      </c>
+      <c r="H46" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I46" s="22">
+        <v>24.130348768799994</v>
+      </c>
+      <c r="J46" s="24">
+        <f t="shared" si="11"/>
+        <v>-0.45478495440000444</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14">
+      <c r="A47" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B47">
+        <v>8</v>
+      </c>
+      <c r="C47">
+        <v>23.0153</v>
+      </c>
+      <c r="D47">
+        <v>23.0153</v>
+      </c>
+      <c r="E47">
+        <v>48.357500000000002</v>
+      </c>
+      <c r="F47" s="16">
+        <f t="shared" si="10"/>
+        <v>25.291312862400002</v>
+      </c>
+      <c r="G47">
+        <v>21</v>
+      </c>
+      <c r="H47" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I47" s="22">
+        <v>25.307081135999997</v>
+      </c>
+      <c r="J47" s="24">
+        <f t="shared" si="11"/>
+        <v>1.5768273599995553E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14">
+      <c r="A48" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B48">
+        <v>9</v>
+      </c>
+      <c r="C48">
+        <v>22.7776</v>
+      </c>
+      <c r="D48">
+        <v>22.7776</v>
+      </c>
+      <c r="E48">
+        <v>47.615699999999997</v>
+      </c>
+      <c r="F48" s="16">
+        <f t="shared" si="10"/>
+        <v>24.788225095199998</v>
+      </c>
+      <c r="G48">
+        <v>21</v>
+      </c>
+      <c r="H48" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I48" s="22">
+        <v>25.235924306400001</v>
+      </c>
+      <c r="J48" s="24">
+        <f t="shared" si="11"/>
+        <v>0.44769921120000333</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10">
+      <c r="A49" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B49">
+        <v>5131</v>
+      </c>
+      <c r="C49">
+        <v>22.698899999999998</v>
+      </c>
+      <c r="D49">
+        <v>22.698899999999998</v>
+      </c>
+      <c r="E49">
+        <v>47.903799999999997</v>
+      </c>
+      <c r="F49" s="16">
+        <f t="shared" si="10"/>
+        <v>25.154288560799998</v>
+      </c>
+      <c r="G49">
+        <v>21</v>
+      </c>
+      <c r="H49" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I49" s="17">
+        <v>25.16</v>
+      </c>
+      <c r="J49" s="24">
+        <f t="shared" si="11"/>
+        <v>5.7114392000023884E-3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10">
+      <c r="A50" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B50">
+        <v>5155</v>
+      </c>
+      <c r="C50">
+        <v>21.792100000000001</v>
+      </c>
+      <c r="D50">
+        <v>21.792100000000001</v>
+      </c>
+      <c r="E50">
+        <v>46.797800000000002</v>
+      </c>
+      <c r="F50" s="16">
+        <f t="shared" si="10"/>
+        <v>24.955488554400002</v>
+      </c>
+      <c r="G50">
+        <v>21</v>
+      </c>
+      <c r="H50" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I50" s="17">
+        <v>24.97</v>
+      </c>
+      <c r="J50" s="24">
+        <f t="shared" si="11"/>
+        <v>1.451144559999662E-2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10">
+      <c r="A51" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B51">
+        <v>5167</v>
+      </c>
+      <c r="C51">
+        <v>21.615500000000001</v>
+      </c>
+      <c r="D51">
+        <v>21.615500000000001</v>
+      </c>
+      <c r="E51">
+        <v>46.652700000000003</v>
+      </c>
+      <c r="F51" s="16">
+        <f t="shared" si="10"/>
+        <v>24.986925302400003</v>
+      </c>
+      <c r="G51">
+        <v>21</v>
+      </c>
+      <c r="H51" s="12">
+        <v>0.99799199999999999</v>
+      </c>
+      <c r="I51" s="17">
+        <v>24.99</v>
+      </c>
+      <c r="J51" s="24">
+        <f t="shared" si="11"/>
+        <v>3.0746975999953463E-3</v>
       </c>
     </row>
   </sheetData>
@@ -1522,22 +2584,22 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="10" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -1667,7 +2729,7 @@
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="19">
+      <c r="A8" s="18">
         <v>5155</v>
       </c>
       <c r="B8" s="4">
@@ -1688,7 +2750,7 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="19">
+      <c r="A9" s="18">
         <v>5167</v>
       </c>
       <c r="B9" s="4">
@@ -1709,7 +2771,7 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="19">
+      <c r="A10" s="18">
         <v>5131</v>
       </c>
       <c r="B10" s="4">
@@ -1730,7 +2792,7 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="18">
+      <c r="A11" s="17">
         <v>7</v>
       </c>
       <c r="D11" s="12">
@@ -1741,7 +2803,7 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="18">
+      <c r="A12" s="17">
         <v>8</v>
       </c>
       <c r="D12" s="12">
@@ -1752,7 +2814,7 @@
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="18">
+      <c r="A13" s="17">
         <v>9</v>
       </c>
       <c r="D13" s="12">
@@ -1788,17 +2850,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="4b0c7577-6c1b-478c-923a-a650d6d013be" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0feec21d-23b4-4c00-874b-59d5ed798470">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010099C27785EF916B49928F172402C7A269" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c7a9e26b68c7148b1f4c19027baf6be7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0feec21d-23b4-4c00-874b-59d5ed798470" xmlns:ns3="4b0c7577-6c1b-478c-923a-a650d6d013be" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ea92f46ce11959a32adf5425306acb8a" ns2:_="" ns3:_="">
     <xsd:import namespace="0feec21d-23b4-4c00-874b-59d5ed798470"/>
@@ -1987,14 +3038,25 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="4b0c7577-6c1b-478c-923a-a650d6d013be" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0feec21d-23b4-4c00-874b-59d5ed798470">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{302BE274-239F-4210-B6F1-3B6D414AB4AC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5356C2EF-818F-45C2-8C57-0949C45041D0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F53A144E-2CA0-4427-89A0-7DEEA1858790}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F53A144E-2CA0-4427-89A0-7DEEA1858790}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5356C2EF-818F-45C2-8C57-0949C45041D0}"/>
 </file>
</xml_diff>